<commit_message>
docs: unify allocation contract hierarchy and eliminate terminology conflict
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_System_Specification.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_System_Specification.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -669,29 +669,29 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2. The 3-Step Priority Order</t>
+          <t>2. Rate Determination Order (Allocation Contract Terms)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Priority Level</t>
+          <t>Rate Determination Level</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Check Condition</t>
+          <t>Contract Condition</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Action Taken</t>
+          <t>Billing Action</t>
         </is>
       </c>
     </row>
@@ -703,17 +703,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Special Partner Deal</t>
+          <t>Custom Negotiated Terms (Operator / Partner)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Does this driver or operator have a special agreed rate in sheet_rental_partners?</t>
+          <t>Does this vehicle's allocation contract specify custom fixed terms in core_rent?</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Charge their special negotiated daily rent and indemnity directly (e.g. Kareem ₹900, Khaja ₹970).</t>
+          <t>Apply the negotiated daily rent and indemnity directly (e.g. Kareem ₹900, Khaja ₹970, Qadir ₹1,070).</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Is the driver in Bengaluru on an individual Uber plan doing 1 or more Ola trips?</t>
+          <t>Is the driver on an individual Uber plan doing 1 or more Ola trips in Bengaluru?</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -747,17 +747,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Standard Trip Slabs</t>
+          <t>Standard Rate Slabs (Allocation Plan)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>If normal driver: Look up city, car model, and completed weekly Uber trips in sheet_rental_slabs.</t>
+          <t>If on standard terms: What plan was agreed when the vehicle was allocated to the driver?</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Apply the rate for that trip tier (e.g. 75+ trips = ₹869/day for Bengaluru WagonR).</t>
+          <t>Match completed weekly trips against city rate card milestones in sheet_rental_slabs (or apply flat rate).</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Base Rate Fallback</t>
+          <t>City Base Fallback</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Apply standard city base rate (WagonR ₹1050, Dzire ₹1200, EV ₹1300, Xcent ₹900).</t>
+          <t>Apply standard city base rate (WagonR ₹1,050, Dzire ₹1,200, EV ₹1,300, Xcent ₹900).</t>
         </is>
       </c>
     </row>
@@ -908,83 +908,100 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Zero-Trip Days</t>
+          <t>Allocation vs Onboarding</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Driver has car but did 0 trips</t>
+          <t>Contract established at Vehicle Allocation</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Rent is charged normally unless car is in maintenance or an approved adjustment is made.</t>
+          <t>Terms chosen when taking delivery of vehicle (core_rent) form the binding legal contract, superseding preliminary onboarding application.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Mid-Week Plan Changes</t>
+          <t>Zero-Trip Days</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Driver wants to switch plan mid-week</t>
+          <t>Driver has car but did 0 trips</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Changes take effect from the start of the next week (coming Monday).</t>
+          <t>Rent is charged normally unless car is in maintenance or an approved adjustment is made.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Mid-Week Allocation</t>
+          <t>Mid-Week Plan Changes</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Driver starts mid-week (e.g. Wednesday)</t>
+          <t>Driver wants to switch plan mid-week</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Calculated pro-rata daily based on active days.</t>
+          <t>Changes take effect from the start of the next week (coming Monday).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Maintenance &amp; Breakdown</t>
+          <t>Mid-Week Allocation</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Car in workshop / off-road</t>
+          <t>Driver starts mid-week (e.g. Wednesday)</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Always ₹0 rent and ₹0 indemnity when billable_rent_day = FALSE in core_daily_vehicle_status.</t>
+          <t>Calculated pro-rata daily based on active days.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t>Maintenance &amp; Breakdown</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Car in workshop / off-road</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Always ₹0 rent and ₹0 indemnity when billable_rent_day = FALSE in core_daily_vehicle_status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>Vehicle Age Discount</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Car crosses age milestone mid-contract</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Discount remains frozen during the active agreement tenure.</t>
         </is>

</xml_diff>